<commit_message>
Correct the marketplace aisle name: SBIR/STTR Aisle, not "Silver Aisle"
The v1 script said "CDAO Tradewinds Silver Aisle." No such aisle exists —
it is the SBIR/STTR Aisle of the Tradewinds Solutions Marketplace. The
narration's "silver aisle" was the script being read accurately, so this
is a Shot 19 re-record and a CTA card re-render, not a pronunciation note.

Fixed in the storyboard script, on-screen text and VO notes, plus the shot
list, editor packet, video-master README, both build scripts, the alignment
doc and the compliance checklist.

Refs: https://www.tradewindai.com/sbir-sttr-aisle
      https://www.tradewindai.com/tw-marketplace

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SGXq8xuRe2C9eXKQfGZQcT
</commit_message>
<xml_diff>
--- a/docs/fm-future-storyboard.xlsx
+++ b/docs/fm-future-storyboard.xlsx
@@ -1214,17 +1214,17 @@
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Find Financial Management of the Future on the CDAO Tradewinds Silver Aisle. Bring your hardest reconciliation and your messiest records — we'll show you what the agents do with them.</t>
+          <t>Find Financial Management of the Future on the CDAO Tradewinds Solutions Marketplace, in the SBIR Aisle. Bring your hardest reconciliation and your messiest records — we'll show you what the agents do with them.</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>Find us on the CDAO Tradewinds Silver Aisle   ·   [POC NAME] · [poc email] · [Innovation Hub link / QR]</t>
+          <t>Find us on the CDAO Tradewinds Solutions Marketplace · SBIR/STTR Aisle   ·   [POC NAME] · [poc email] · [Innovation Hub link / QR]</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>CTA card; POC name + email and Silver Aisle or Innovation Hub link/QR. Replace the generic poc@guidehouse.com placeholder with the named POC before final render.</t>
+          <t>CTA card; POC name + email and the Tradewinds Solutions Marketplace / SBIR-STTR Aisle link or QR. Replace the generic poc@guidehouse.com placeholder with the named POC before final render. On-screen text must read SBIR/STTR Aisle — there is no 'Silver Aisle'.</t>
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
-          <t>"Silver Aisle" here is the CDAO Tradewinds marketplace aisle — it is the correct term and NOT a mispronunciation of SBIR. Read it plainly: "the CDAO Tradewinds Silver Aisle." If this line is re-recorded, keep the wording.</t>
+          <t>CORRECTION (Jul 2026): the v1 script said "Silver Aisle" — that aisle does not exist. The correct name is the CDAO Tradewinds Solutions Marketplace SBIR/STTR Aisle (commonly "SBIR Aisle"). PRONUNCIATION: same as Shot 17 — SBIR is said as a word, "SY-ber," so this reads "the SY-ber aisle." Do NOT spell it S-B-I-R.</t>
         </is>
       </c>
     </row>

</xml_diff>